<commit_message>
Removing the solution of last years labs
</commit_message>
<xml_diff>
--- a/Teaching/course_schedule.xlsx
+++ b/Teaching/course_schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hakim/git/mywebsite/hqahtan.github.io/Teaching/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759C5EF3-C8D9-764C-B2F8-B579E2FD42AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90BA8C3B-7E35-0640-85FD-362C85579C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1800" yWindow="620" windowWidth="34280" windowHeight="19560" xr2:uid="{72E94DF8-02B7-44D7-9115-6D7B922CAFF9}"/>
   </bookViews>
@@ -317,81 +317,45 @@
     <t>https://hqahtan.github.io/Teaching/lectures/week_1/2_DataModels.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_1/2_DataModels/2_DataModels_answers_2738.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_2/1_DE_1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_2/1_DE_1/1_DE_1_answers_1063.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_2/2_DE_2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_2/2_DE_2/2_DE_2_answers_6271.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_2/3_ICs.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_2/3_ICs/3_ICs_answers_3592.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_3/1_FDs.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_3/1_FDs/1_FDs_answers_0372.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_3/Social.html</t>
   </si>
   <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_3/2_Indexing_DI.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_3/2_Indexing_DI/2_Indexing_DI_answers_6021.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_3/3_HDA_SS.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_3/3_HDA_SS/3_HDA_SS_answers_5529.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_4/1_DP1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_4/1_DP1/1_DP1_answers_8190.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/assignments/assignment_1.html</t>
   </si>
   <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_4/2_DP2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_4/2_DP2/2_DP2_answers_8826.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_4/3_visualization_1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_4/3_data_visualization_1/data_visualization_1_answers.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_5/1_visualization_2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_5/1_data_visualization_2/data_visualization_2_answers_a20f95b.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_5/2_regression_1_redacted.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_5/2_supervised_1/supervised_1_answers_34b1c2a.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/exams/Mid-TermExam.html</t>
   </si>
   <si>
@@ -407,73 +371,109 @@
     <t>https://hqahtan.github.io/Teaching/lectures/week_6/2_regression_3.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_6/2_supervised_3/supervised_3_answers_3ba2fbb.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_6/3_deep_learning.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_6/3_deep_learning/supervised_4_answers_3gh12s.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_7/1_missing_data_1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_7/1_missing_data_1/missing_data_1_answers_ej4ab45.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_7/2_missing_data_2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_7/2_missing_data_2/missing_data_2_answers_32ksaae.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_7/3_clustering_1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_7/3_clustering_1/clustering_1_answers_a23b1e3.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_8/1_clustering_2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_8/1_clustering_2/clustering_2_answers_25ae1b.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_8/2_text_mining_1.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_8/2_text_mining_1/text_mining_1_answers_655643.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_8/3_text_mining_2.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_8/3_text_mining_2/text_mining_2_answers_3b2f11.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_9/1_TS.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_9/1_TS/1_TS_answers_9022.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_9/2_DS.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_9/2_DS/2_DS_answers_0186.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/lectures/week_9/3_Fairness.pdf</t>
   </si>
   <si>
-    <t>https://hqahtan.github.io/Teaching/labs/week_9/3_Fairness/3_Fairness_answers_6781.html</t>
-  </si>
-  <si>
     <t>https://hqahtan.github.io/Teaching/assignments/assignment_4.html</t>
   </si>
   <si>
     <t>https://hqahtan.github.io/Teaching/exams/FinalExam.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/3_Fairness/3_Fairness.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/2_DS/2_DS.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/1_TS/1_TS.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/3_text_mining_2/text_mining_2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/2_text_mining_1/text_mining_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/1_clustering_2/clustering_2_answers.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/3_clustering_1/clustering_1_answers.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/2_missing_data_2/missing_data_2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/1_missing_data_1/missing_data_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_6/3_deep_learning/supervised_4.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_6/2_supervised_3/supervised_3.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_5/2_supervised_1/supervised_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_5/1_data_visualization_2/data_visualization_2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/3_data_visualization_1/data_visualization_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/2_DP2/2_DP2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/1_DP1/1_DP1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/3_HDA_SS/3_HDA_SS.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/2_Indexing_DI/2_Indexing_DI.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/1_FDs/1_FDs.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/3_ICs/3_ICs.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/2_DE_2/2_DE_2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/1_DE_1/1_DE_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_1/2_DataModels/2_DataModels.html</t>
   </si>
 </sst>
 </file>
@@ -971,7 +971,7 @@
         <v>39</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -988,7 +988,7 @@
         <v>40</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>31</v>
@@ -1009,7 +1009,7 @@
         <v>40</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>94</v>
+        <v>143</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1027,7 +1027,7 @@
         <v>77</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>68</v>
@@ -1048,7 +1048,7 @@
         <v>77</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>96</v>
+        <v>142</v>
       </c>
       <c r="I9" s="4"/>
     </row>
@@ -1066,7 +1066,7 @@
         <v>41</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>12</v>
@@ -1087,7 +1087,7 @@
         <v>41</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="I11" s="4"/>
     </row>
@@ -1105,7 +1105,7 @@
         <v>73</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>14</v>
@@ -1126,7 +1126,7 @@
         <v>73</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="I13" s="4"/>
     </row>
@@ -1144,7 +1144,7 @@
         <v>76</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>75</v>
@@ -1183,7 +1183,7 @@
         <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
       <c r="I16" s="4"/>
     </row>
@@ -1201,7 +1201,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>13</v>
@@ -1222,7 +1222,7 @@
         <v>63</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="I18" s="4"/>
     </row>
@@ -1240,7 +1240,7 @@
         <v>42</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>69</v>
@@ -1261,7 +1261,7 @@
         <v>42</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
       <c r="I20" s="4"/>
     </row>
@@ -1279,7 +1279,7 @@
         <v>79</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I21" s="4"/>
     </row>
@@ -1297,7 +1297,7 @@
         <v>43</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>70</v>
@@ -1318,7 +1318,7 @@
         <v>43</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="I23" s="4"/>
     </row>
@@ -1336,7 +1336,7 @@
         <v>64</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>87</v>
@@ -1357,7 +1357,7 @@
         <v>65</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="I25" s="4"/>
     </row>
@@ -1375,7 +1375,7 @@
         <v>44</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>87</v>
@@ -1396,7 +1396,7 @@
         <v>45</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="I27" s="4"/>
     </row>
@@ -1414,7 +1414,7 @@
         <v>46</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>66</v>
@@ -1435,7 +1435,7 @@
         <v>47</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="I29" s="4"/>
     </row>
@@ -1485,7 +1485,7 @@
         <v>86</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="I32" s="4"/>
     </row>
@@ -1503,7 +1503,7 @@
         <v>78</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="I33" s="4"/>
     </row>
@@ -1521,7 +1521,7 @@
         <v>48</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>67</v>
@@ -1542,7 +1542,7 @@
         <v>48</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="I35" s="4"/>
     </row>
@@ -1560,7 +1560,7 @@
         <v>49</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>19</v>
@@ -1581,7 +1581,7 @@
         <v>49</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="I37" s="4"/>
     </row>
@@ -1599,7 +1599,7 @@
         <v>50</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>20</v>
@@ -1620,7 +1620,7 @@
         <v>50</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="I39" s="4"/>
     </row>
@@ -1638,7 +1638,7 @@
         <v>51</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>21</v>
@@ -1659,7 +1659,7 @@
         <v>52</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="I41" s="4"/>
     </row>
@@ -1677,7 +1677,7 @@
         <v>53</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>21</v>
@@ -1698,7 +1698,7 @@
         <v>54</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I43" s="4"/>
     </row>
@@ -1716,7 +1716,7 @@
         <v>55</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>22</v>
@@ -1737,7 +1737,7 @@
         <v>55</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I45" s="4"/>
     </row>
@@ -1755,7 +1755,7 @@
         <v>80</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="I46" s="4"/>
     </row>
@@ -1773,7 +1773,7 @@
         <v>56</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>23</v>
@@ -1794,7 +1794,7 @@
         <v>57</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="I48" s="4"/>
     </row>
@@ -1812,7 +1812,7 @@
         <v>58</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>24</v>
@@ -1833,7 +1833,7 @@
         <v>58</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="I50" s="4"/>
     </row>
@@ -1869,7 +1869,7 @@
         <v>59</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>24</v>
@@ -1890,7 +1890,7 @@
         <v>59</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="I53" s="4"/>
     </row>
@@ -1908,7 +1908,7 @@
         <v>60</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>17</v>
@@ -1929,7 +1929,7 @@
         <v>60</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="I55" s="4"/>
     </row>
@@ -1947,7 +1947,7 @@
         <v>61</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>30</v>
@@ -1968,7 +1968,7 @@
         <v>61</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="I57" s="4"/>
     </row>
@@ -1986,7 +1986,7 @@
         <v>62</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>18</v>
@@ -2007,7 +2007,7 @@
         <v>62</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="I59" s="4"/>
     </row>
@@ -2025,7 +2025,7 @@
         <v>81</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="I60" s="4"/>
     </row>
@@ -2075,7 +2075,7 @@
         <v>85</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="I63" s="4"/>
     </row>

</xml_diff>